<commit_message>
Finalize manuscript outputs: Table 3, Table 4, Table S1, pooled meta
Checkpoint of the state the finished manuscript was written against.

- Add scripts/table3_gapmap.py, table4_ae_safety.py, table_s1_references.py
  and pooled_meta.py, plus their outputs in tables/.
- Rename the observational AE table to ae_events_observational.csv so the two
  pipelines' event files are distinguishable where table4_ae_safety.py joins
  them.
- Add observational_studies/overrides.json and the Noller ibogaine PDF.
- Refresh all condition tables, figures and cleaned datasets from the current
  clinical_master.csv, and apply the Prior 2014 removal to the manuscript.
</commit_message>
<xml_diff>
--- a/clinical_trials/outputs/clinical_master.xlsx
+++ b/clinical_trials/outputs/clinical_master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BT50"/>
+  <dimension ref="A1:BU50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -709,70 +709,75 @@
       </c>
       <c r="BG1" t="inlineStr">
         <is>
+          <t>BaseStatusReportedYN</t>
+        </is>
+      </c>
+      <c r="BH1" t="inlineStr">
+        <is>
           <t>SafetyReported</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>AnyAEReported</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>NumDistinctAEs</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>NParticipantsWithAE</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>AE_denominator</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>ArmScope</t>
         </is>
       </c>
-      <c r="BM1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>WorstSeverity</t>
         </is>
       </c>
-      <c r="BN1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>text_source</t>
         </is>
       </c>
-      <c r="BO1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>text_format</t>
         </is>
       </c>
-      <c r="BP1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="BQ1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>PromptVersion</t>
         </is>
       </c>
-      <c r="BR1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>RubricVersion</t>
         </is>
       </c>
-      <c r="BS1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>Temperature</t>
         </is>
       </c>
-      <c r="BT1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>SourcePDF</t>
         </is>
@@ -979,64 +984,69 @@
       </c>
       <c r="BG2" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH2" t="inlineStr">
+      <c r="BI2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI2" t="n">
+      <c r="BJ2" t="n">
         <v>4</v>
       </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK2" t="n">
+      <c r="BK2" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL2" t="n">
         <v>10</v>
       </c>
-      <c r="BL2" t="inlineStr">
+      <c r="BM2" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM2" t="inlineStr">
+      <c r="BN2" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN2" t="inlineStr">
+      <c r="BO2" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO2" t="inlineStr">
+      <c r="BP2" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP2" t="inlineStr">
+      <c r="BQ2" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ2" t="inlineStr">
+      <c r="BR2" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR2" t="inlineStr">
+      <c r="BS2" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT2" t="inlineStr">
+      <c r="BT2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU2" t="inlineStr">
         <is>
           <t>alcohol/Psilocybin-assisted treatment for alcohol dependence - A proof-of-concept study (Bogenschutz et al., 2015) (1).pdf</t>
         </is>
@@ -1241,66 +1251,71 @@
       </c>
       <c r="BG3" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH3" t="inlineStr">
+      <c r="BI3" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI3" t="inlineStr">
+      <c r="BJ3" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK3" t="n">
+      <c r="BK3" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL3" t="n">
         <v>93</v>
       </c>
-      <c r="BL3" t="inlineStr">
+      <c r="BM3" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM3" t="inlineStr">
+      <c r="BN3" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN3" t="inlineStr">
+      <c r="BO3" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO3" t="inlineStr">
+      <c r="BP3" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP3" t="inlineStr">
+      <c r="BQ3" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ3" t="inlineStr">
+      <c r="BR3" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR3" t="inlineStr">
+      <c r="BS3" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS3" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT3" t="inlineStr">
+      <c r="BT3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU3" t="inlineStr">
         <is>
           <t>alcohol/jamapsychiatry_bogenschutz_2022_oi_220046_1664208846.29988 (1).pdf</t>
         </is>
@@ -1519,68 +1534,73 @@
       </c>
       <c r="BG4" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH4" t="inlineStr">
+      <c r="BI4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI4" t="inlineStr">
+      <c r="BJ4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ4" t="inlineStr">
+      <c r="BK4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK4" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL4" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM4" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM4" t="inlineStr">
+      <c r="BN4" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN4" t="inlineStr">
+      <c r="BO4" t="inlineStr">
         <is>
           <t>OCR</t>
         </is>
       </c>
-      <c r="BO4" t="inlineStr">
+      <c r="BP4" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="BP4" t="inlineStr">
+      <c r="BQ4" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ4" t="inlineStr">
+      <c r="BR4" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR4" t="inlineStr">
+      <c r="BS4" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS4" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT4" t="inlineStr">
+      <c r="BT4" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU4" t="inlineStr">
         <is>
           <t>alcohol/Bowen, W. T., Soskin, R. A., &amp; Chotlos, J. W. (1970) Lysergic acid diethylamide.pdf</t>
         </is>
@@ -1799,66 +1819,71 @@
       </c>
       <c r="BG5" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BH5" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH5" t="inlineStr">
+      <c r="BI5" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI5" t="n">
+      <c r="BJ5" t="n">
         <v>7</v>
       </c>
-      <c r="BJ5" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BK5" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL5" t="inlineStr">
+        <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BL5" t="inlineStr">
+      <c r="BM5" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM5" t="inlineStr">
+      <c r="BN5" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN5" t="inlineStr">
+      <c r="BO5" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO5" t="inlineStr">
+      <c r="BP5" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP5" t="inlineStr">
+      <c r="BQ5" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ5" t="inlineStr">
+      <c r="BR5" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR5" t="inlineStr">
+      <c r="BS5" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS5" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT5" t="inlineStr">
+      <c r="BT5" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU5" t="inlineStr">
         <is>
           <t>alcohol/costello-1969-an-evaluation-of-aversion-and-lsd-therapy-in-the-treatment-of-alcoholism.pdf</t>
         </is>
@@ -2067,64 +2092,69 @@
       </c>
       <c r="BG6" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH6" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH6" t="inlineStr">
+      <c r="BI6" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI6" t="n">
+      <c r="BJ6" t="n">
         <v>4</v>
       </c>
-      <c r="BJ6" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK6" t="n">
+      <c r="BK6" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL6" t="n">
         <v>40</v>
       </c>
-      <c r="BL6" t="inlineStr">
+      <c r="BM6" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM6" t="inlineStr">
+      <c r="BN6" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN6" t="inlineStr">
+      <c r="BO6" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO6" t="inlineStr">
+      <c r="BP6" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP6" t="inlineStr">
+      <c r="BQ6" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ6" t="inlineStr">
+      <c r="BR6" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR6" t="inlineStr">
+      <c r="BS6" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS6" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT6" t="inlineStr">
+      <c r="BT6" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU6" t="inlineStr">
         <is>
           <t>alcohol/dakwar-et-al-2019-a-single-ketamine-infusion-combined-with-motivational-enhancement-therapy-for-alcohol-use-disorder-a (1).pdf</t>
         </is>
@@ -2337,68 +2367,73 @@
       </c>
       <c r="BG7" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH7" t="inlineStr">
+      <c r="BI7" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI7" t="inlineStr">
+      <c r="BJ7" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ7" t="inlineStr">
+      <c r="BK7" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK7" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL7" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM7" t="inlineStr">
+      <c r="BN7" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN7" t="inlineStr">
+      <c r="BO7" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO7" t="inlineStr">
+      <c r="BP7" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP7" t="inlineStr">
+      <c r="BQ7" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ7" t="inlineStr">
+      <c r="BR7" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR7" t="inlineStr">
+      <c r="BS7" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS7" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT7" t="inlineStr">
+      <c r="BT7" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU7" t="inlineStr">
         <is>
           <t>alcohol/s41467-019-13162-w.pdf</t>
         </is>
@@ -2615,68 +2650,73 @@
       </c>
       <c r="BG8" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH8" t="inlineStr">
+      <c r="BI8" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI8" t="inlineStr">
+      <c r="BJ8" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ8" t="inlineStr">
+      <c r="BK8" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK8" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL8" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM8" t="inlineStr">
+      <c r="BN8" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN8" t="inlineStr">
+      <c r="BO8" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO8" t="inlineStr">
+      <c r="BP8" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="BP8" t="inlineStr">
+      <c r="BQ8" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ8" t="inlineStr">
+      <c r="BR8" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR8" t="inlineStr">
+      <c r="BS8" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS8" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT8" t="inlineStr">
+      <c r="BT8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU8" t="inlineStr">
         <is>
           <t>alcohol/Denson, R., &amp; Sydiaha, D. (1970) A controlled study of LSD treatment in alcoholism.pdf</t>
         </is>
@@ -2895,62 +2935,67 @@
       </c>
       <c r="BG9" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH9" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH9" t="inlineStr">
+      <c r="BI9" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
-      </c>
-      <c r="BI9" t="n">
-        <v>3</v>
       </c>
       <c r="BJ9" t="n">
         <v>3</v>
       </c>
       <c r="BK9" t="n">
+        <v>3</v>
+      </c>
+      <c r="BL9" t="n">
         <v>71</v>
       </c>
-      <c r="BL9" t="inlineStr">
+      <c r="BM9" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM9" t="inlineStr">
+      <c r="BN9" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN9" t="inlineStr">
+      <c r="BO9" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO9" t="inlineStr">
+      <c r="BP9" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP9" t="inlineStr">
+      <c r="BQ9" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ9" t="inlineStr">
+      <c r="BR9" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR9" t="inlineStr">
+      <c r="BS9" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS9" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT9" t="inlineStr">
+      <c r="BT9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU9" t="inlineStr">
         <is>
           <t>alcohol/qjsa.1967.28.295.pdf</t>
         </is>
@@ -3163,68 +3208,73 @@
       </c>
       <c r="BG10" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH10" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH10" t="inlineStr">
+      <c r="BI10" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI10" t="inlineStr">
+      <c r="BJ10" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ10" t="inlineStr">
+      <c r="BK10" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK10" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL10" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM10" t="inlineStr">
+      <c r="BN10" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN10" t="inlineStr">
+      <c r="BO10" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO10" t="inlineStr">
+      <c r="BP10" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP10" t="inlineStr">
+      <c r="BQ10" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ10" t="inlineStr">
+      <c r="BR10" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR10" t="inlineStr">
+      <c r="BS10" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS10" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT10" t="inlineStr">
+      <c r="BT10" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU10" t="inlineStr">
         <is>
           <t>alcohol/10.1177_02698811241254834.pdf</t>
         </is>
@@ -3435,64 +3485,69 @@
       </c>
       <c r="BG11" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH11" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH11" t="inlineStr">
+      <c r="BI11" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI11" t="inlineStr">
+      <c r="BJ11" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ11" t="n">
+      <c r="BK11" t="n">
         <v>20</v>
       </c>
-      <c r="BK11" t="n">
+      <c r="BL11" t="n">
         <v>96</v>
       </c>
-      <c r="BL11" t="inlineStr">
+      <c r="BM11" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM11" t="inlineStr">
+      <c r="BN11" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN11" t="inlineStr">
+      <c r="BO11" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO11" t="inlineStr">
+      <c r="BP11" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP11" t="inlineStr">
+      <c r="BQ11" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ11" t="inlineStr">
+      <c r="BR11" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR11" t="inlineStr">
+      <c r="BS11" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS11" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT11" t="inlineStr">
+      <c r="BT11" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU11" t="inlineStr">
         <is>
           <t>alcohol/grabski-et-al-2022-adjunctive-ketamine-with-relapse-prevention-based-psychological-therapy-in-the-treatment-of-alcohol (1).pdf</t>
         </is>
@@ -3701,64 +3756,69 @@
       </c>
       <c r="BG12" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH12" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH12" t="inlineStr">
+      <c r="BI12" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI12" t="n">
+      <c r="BJ12" t="n">
         <v>23</v>
       </c>
-      <c r="BJ12" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK12" t="n">
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL12" t="n">
         <v>20</v>
       </c>
-      <c r="BL12" t="inlineStr">
+      <c r="BM12" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM12" t="inlineStr">
+      <c r="BN12" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN12" t="inlineStr">
+      <c r="BO12" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO12" t="inlineStr">
+      <c r="BP12" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP12" t="inlineStr">
+      <c r="BQ12" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ12" t="inlineStr">
+      <c r="BR12" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR12" t="inlineStr">
+      <c r="BS12" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS12" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT12" t="inlineStr">
+      <c r="BT12" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU12" t="inlineStr">
         <is>
           <t>alcohol/Heinzerling, K. G., Sergi,. Nature-themed video intervention.pdf</t>
         </is>
@@ -3969,64 +4029,69 @@
       </c>
       <c r="BG13" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH13" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH13" t="inlineStr">
+      <c r="BI13" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI13" t="n">
+      <c r="BJ13" t="n">
         <v>5</v>
       </c>
-      <c r="BJ13" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK13" t="n">
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL13" t="n">
         <v>72</v>
       </c>
-      <c r="BL13" t="inlineStr">
+      <c r="BM13" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM13" t="inlineStr">
+      <c r="BN13" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN13" t="inlineStr">
+      <c r="BO13" t="inlineStr">
         <is>
           <t>OCR</t>
         </is>
       </c>
-      <c r="BO13" t="inlineStr">
+      <c r="BP13" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="BP13" t="inlineStr">
+      <c r="BQ13" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ13" t="inlineStr">
+      <c r="BR13" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR13" t="inlineStr">
+      <c r="BS13" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS13" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT13" t="inlineStr">
+      <c r="BT13" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU13" t="inlineStr">
         <is>
           <t>alcohol/Hollister, L. E., Shelton, J., &amp; Krieger, G. (1969). A controlled comparison of lysergic acid diethylamide (LSD).pdf</t>
         </is>
@@ -4239,66 +4304,71 @@
       </c>
       <c r="BG14" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH14" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH14" t="inlineStr">
+      <c r="BI14" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI14" t="n">
+      <c r="BJ14" t="n">
         <v>5</v>
       </c>
-      <c r="BJ14" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BK14" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL14" t="inlineStr">
+        <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BL14" t="inlineStr">
+      <c r="BM14" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM14" t="inlineStr">
+      <c r="BN14" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN14" t="inlineStr">
+      <c r="BO14" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO14" t="inlineStr">
+      <c r="BP14" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP14" t="inlineStr">
+      <c r="BQ14" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ14" t="inlineStr">
+      <c r="BR14" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR14" t="inlineStr">
+      <c r="BS14" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS14" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT14" t="inlineStr">
+      <c r="BT14" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU14" t="inlineStr">
         <is>
           <t>alcohol/Jensen, S. E., &amp; Ramsay, R. (1963). Treatment of chronic alcoholism with lysergic acid diethylamide.pdf</t>
         </is>
@@ -4505,66 +4575,71 @@
       </c>
       <c r="BG15" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH15" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH15" t="inlineStr">
+      <c r="BI15" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI15" t="inlineStr">
+      <c r="BJ15" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ15" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK15" t="n">
+      <c r="BK15" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL15" t="n">
         <v>10</v>
       </c>
-      <c r="BL15" t="inlineStr">
+      <c r="BM15" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM15" t="inlineStr">
+      <c r="BN15" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN15" t="inlineStr">
+      <c r="BO15" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO15" t="inlineStr">
+      <c r="BP15" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP15" t="inlineStr">
+      <c r="BQ15" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ15" t="inlineStr">
+      <c r="BR15" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR15" t="inlineStr">
+      <c r="BS15" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS15" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT15" t="inlineStr">
+      <c r="BT15" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU15" t="inlineStr">
         <is>
           <t>alcohol/v1_covered_0fc93b81-dfaa-4726-85f8-e5a38067a1dc (1).pdf</t>
         </is>
@@ -4777,68 +4852,73 @@
       </c>
       <c r="BG16" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH16" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH16" t="inlineStr">
+      <c r="BI16" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI16" t="inlineStr">
+      <c r="BJ16" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ16" t="inlineStr">
+      <c r="BK16" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK16" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL16" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM16" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM16" t="inlineStr">
+      <c r="BN16" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN16" t="inlineStr">
+      <c r="BO16" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO16" t="inlineStr">
+      <c r="BP16" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP16" t="inlineStr">
+      <c r="BQ16" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ16" t="inlineStr">
+      <c r="BR16" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR16" t="inlineStr">
+      <c r="BS16" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS16" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT16" t="inlineStr">
+      <c r="BT16" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU16" t="inlineStr">
         <is>
           <t>alcohol/Johnson, F. G. (1969). LSD in the treatment of alcoholism.pdf</t>
         </is>
@@ -5051,62 +5131,67 @@
       </c>
       <c r="BG17" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH17" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH17" t="inlineStr">
+      <c r="BI17" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI17" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ17" t="n">
         <v>0</v>
       </c>
       <c r="BK17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL17" t="n">
         <v>69</v>
       </c>
-      <c r="BL17" t="inlineStr">
+      <c r="BM17" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM17" t="inlineStr">
+      <c r="BN17" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN17" t="inlineStr">
+      <c r="BO17" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO17" t="inlineStr">
+      <c r="BP17" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP17" t="inlineStr">
+      <c r="BQ17" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ17" t="inlineStr">
+      <c r="BR17" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR17" t="inlineStr">
+      <c r="BS17" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS17" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT17" t="inlineStr">
+      <c r="BT17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU17" t="inlineStr">
         <is>
           <t>alcohol/Kurland, A. A., Unger, S., Shaffer, J. W., &amp; Savage, C. (1967). Psychedelic therapy utilizing LSD in the treatment of the alcoholic patient_ a pre.pdf</t>
         </is>
@@ -5381,68 +5466,73 @@
       </c>
       <c r="BG18" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BH18" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH18" t="inlineStr">
+      <c r="BI18" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI18" t="inlineStr">
+      <c r="BJ18" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ18" t="inlineStr">
+      <c r="BK18" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK18" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL18" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM18" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM18" t="inlineStr">
+      <c r="BN18" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN18" t="inlineStr">
+      <c r="BO18" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO18" t="inlineStr">
+      <c r="BP18" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP18" t="inlineStr">
+      <c r="BQ18" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ18" t="inlineStr">
+      <c r="BR18" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR18" t="inlineStr">
+      <c r="BS18" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS18" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT18" t="inlineStr">
+      <c r="BT18" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU18" t="inlineStr">
         <is>
           <t>alcohol/Ludwig, A., Levine, J., Stark, L., &amp; Lazar, R. (1969) A clinical study of LSD treatment in alcoholism.pdf</t>
         </is>
@@ -5653,62 +5743,67 @@
       </c>
       <c r="BG19" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH19" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH19" t="inlineStr">
+      <c r="BI19" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI19" t="n">
+      <c r="BJ19" t="n">
         <v>19</v>
       </c>
-      <c r="BJ19" t="n">
+      <c r="BK19" t="n">
         <v>16</v>
       </c>
-      <c r="BK19" t="n">
+      <c r="BL19" t="n">
         <v>30</v>
       </c>
-      <c r="BL19" t="inlineStr">
+      <c r="BM19" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM19" t="inlineStr">
+      <c r="BN19" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN19" t="inlineStr">
+      <c r="BO19" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO19" t="inlineStr">
+      <c r="BP19" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP19" t="inlineStr">
+      <c r="BQ19" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ19" t="inlineStr">
+      <c r="BR19" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR19" t="inlineStr">
+      <c r="BS19" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS19" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT19" t="inlineStr">
+      <c r="BT19" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU19" t="inlineStr">
         <is>
           <t>alcohol/Addiction - 2025 - Luquiens - Psilocybin in alcohol use disorder and comorbid depressive symptoms  Results from a.pdf</t>
         </is>
@@ -5919,66 +6014,71 @@
       </c>
       <c r="BG20" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH20" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH20" t="inlineStr">
+      <c r="BI20" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI20" t="n">
+      <c r="BJ20" t="n">
         <v>6</v>
       </c>
-      <c r="BJ20" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BK20" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL20" t="inlineStr">
+        <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BL20" t="inlineStr">
+      <c r="BM20" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM20" t="inlineStr">
+      <c r="BN20" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN20" t="inlineStr">
+      <c r="BO20" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO20" t="inlineStr">
+      <c r="BP20" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP20" t="inlineStr">
+      <c r="BQ20" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ20" t="inlineStr">
+      <c r="BR20" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR20" t="inlineStr">
+      <c r="BS20" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS20" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT20" t="inlineStr">
+      <c r="BT20" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU20" t="inlineStr">
         <is>
           <t>alcohol/MacLean, J. R., MacDonald, D. C., Byrne, U. P., &amp; Hubbard, A. M. (196. The use of LSD-25 in the treatment of alcoholism and other psychiatric problems.pdf</t>
         </is>
@@ -6189,62 +6289,67 @@
       </c>
       <c r="BG21" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH21" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH21" t="inlineStr">
+      <c r="BI21" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI21" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ21" t="n">
         <v>0</v>
       </c>
       <c r="BK21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL21" t="n">
         <v>18</v>
       </c>
-      <c r="BL21" t="inlineStr">
+      <c r="BM21" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM21" t="inlineStr">
+      <c r="BN21" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN21" t="inlineStr">
+      <c r="BO21" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO21" t="inlineStr">
+      <c r="BP21" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP21" t="inlineStr">
+      <c r="BQ21" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ21" t="inlineStr">
+      <c r="BR21" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR21" t="inlineStr">
+      <c r="BS21" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS21" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT21" t="inlineStr">
+      <c r="BT21" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU21" t="inlineStr">
         <is>
           <t>alcohol/Marva. Ketamine Therapy in Patients of Alcohol Use Disorder_ A Prospective Pilot Study to Evaluate Abstinence Rate with This Add-on Treatment Modality.pdf</t>
         </is>
@@ -6455,68 +6560,73 @@
       </c>
       <c r="BG22" t="inlineStr">
         <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="BH22" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH22" t="inlineStr">
+      <c r="BI22" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI22" t="inlineStr">
+      <c r="BJ22" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ22" t="inlineStr">
+      <c r="BK22" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK22" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL22" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM22" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM22" t="inlineStr">
+      <c r="BN22" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN22" t="inlineStr">
+      <c r="BO22" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO22" t="inlineStr">
+      <c r="BP22" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP22" t="inlineStr">
+      <c r="BQ22" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ22" t="inlineStr">
+      <c r="BR22" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR22" t="inlineStr">
+      <c r="BS22" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS22" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT22" t="inlineStr">
+      <c r="BT22" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU22" t="inlineStr">
         <is>
           <t>alcohol/1-s2.0-S037687162200093X-main (1).pdf</t>
         </is>
@@ -6733,21 +6843,21 @@
       </c>
       <c r="BG23" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BH23" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH23" t="inlineStr">
+      <c r="BI23" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI23" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ23" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
+      <c r="BJ23" t="n">
+        <v>0</v>
       </c>
       <c r="BK23" t="inlineStr">
         <is>
@@ -6756,43 +6866,48 @@
       </c>
       <c r="BL23" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM23" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM23" t="inlineStr">
+      <c r="BN23" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN23" t="inlineStr">
+      <c r="BO23" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO23" t="inlineStr">
+      <c r="BP23" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP23" t="inlineStr">
+      <c r="BQ23" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ23" t="inlineStr">
+      <c r="BR23" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR23" t="inlineStr">
+      <c r="BS23" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS23" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT23" t="inlineStr">
+      <c r="BT23" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU23" t="inlineStr">
         <is>
           <t>alcohol/1-s2.0-S1551714422003020-main.pdf</t>
         </is>
@@ -7003,64 +7118,69 @@
       </c>
       <c r="BG24" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH24" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH24" t="inlineStr">
+      <c r="BI24" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI24" t="n">
+      <c r="BJ24" t="n">
         <v>3</v>
       </c>
-      <c r="BJ24" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK24" t="n">
+      <c r="BK24" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL24" t="n">
         <v>68</v>
       </c>
-      <c r="BL24" t="inlineStr">
+      <c r="BM24" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM24" t="inlineStr">
+      <c r="BN24" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN24" t="inlineStr">
+      <c r="BO24" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO24" t="inlineStr">
+      <c r="BP24" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP24" t="inlineStr">
+      <c r="BQ24" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ24" t="inlineStr">
+      <c r="BR24" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR24" t="inlineStr">
+      <c r="BS24" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT24" t="inlineStr">
+      <c r="BT24" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU24" t="inlineStr">
         <is>
           <t>alcohol/o-reilly-funk-1964-lsd-in-chronic-alcoholism.pdf</t>
         </is>
@@ -7269,68 +7389,73 @@
       </c>
       <c r="BG25" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH25" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH25" t="inlineStr">
+      <c r="BI25" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI25" t="inlineStr">
+      <c r="BJ25" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ25" t="inlineStr">
+      <c r="BK25" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK25" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL25" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM25" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM25" t="inlineStr">
+      <c r="BN25" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN25" t="inlineStr">
+      <c r="BO25" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO25" t="inlineStr">
+      <c r="BP25" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP25" t="inlineStr">
+      <c r="BQ25" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ25" t="inlineStr">
+      <c r="BR25" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR25" t="inlineStr">
+      <c r="BS25" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS25" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT25" t="inlineStr">
+      <c r="BT25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU25" t="inlineStr">
         <is>
           <t>alcohol/s41598-024-52967-8.pdf</t>
         </is>
@@ -7543,68 +7668,73 @@
       </c>
       <c r="BG26" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH26" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH26" t="inlineStr">
+      <c r="BI26" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI26" t="inlineStr">
+      <c r="BJ26" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ26" t="inlineStr">
+      <c r="BK26" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK26" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL26" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM26" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM26" t="inlineStr">
+      <c r="BN26" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN26" t="inlineStr">
+      <c r="BO26" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO26" t="inlineStr">
+      <c r="BP26" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP26" t="inlineStr">
+      <c r="BQ26" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ26" t="inlineStr">
+      <c r="BR26" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR26" t="inlineStr">
+      <c r="BS26" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS26" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT26" t="inlineStr">
+      <c r="BT26" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU26" t="inlineStr">
         <is>
           <t>alcohol/pagni-et-al-2025-multidimensional-personality-changes-following-psilocybin-assisted-therapy-in-patients-with-alcohol (1).pdf</t>
         </is>
@@ -7817,64 +7947,69 @@
       </c>
       <c r="BG27" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH27" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH27" t="inlineStr">
+      <c r="BI27" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI27" t="n">
-        <v>1</v>
-      </c>
       <c r="BJ27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK27" t="n">
         <v>2</v>
       </c>
-      <c r="BK27" t="inlineStr">
+      <c r="BL27" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BL27" t="inlineStr">
+      <c r="BM27" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM27" t="inlineStr">
+      <c r="BN27" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN27" t="inlineStr">
+      <c r="BO27" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO27" t="inlineStr">
+      <c r="BP27" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP27" t="inlineStr">
+      <c r="BQ27" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ27" t="inlineStr">
+      <c r="BR27" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR27" t="inlineStr">
+      <c r="BS27" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS27" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT27" t="inlineStr">
+      <c r="BT27" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU27" t="inlineStr">
         <is>
           <t>alcohol/Pahnke, W. N., Kurland, A. A., Unger, S., Savage, C., &amp; Grof, S. (1970). The experimental use of psychedelic (LSD) psychotherapy.pdf</t>
         </is>
@@ -8079,66 +8214,71 @@
       </c>
       <c r="BG28" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH28" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH28" t="inlineStr">
+      <c r="BI28" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI28" t="inlineStr">
+      <c r="BJ28" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ28" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK28" t="n">
+      <c r="BK28" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL28" t="n">
         <v>40</v>
       </c>
-      <c r="BL28" t="inlineStr">
+      <c r="BM28" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM28" t="inlineStr">
+      <c r="BN28" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN28" t="inlineStr">
+      <c r="BO28" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO28" t="inlineStr">
+      <c r="BP28" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP28" t="inlineStr">
+      <c r="BQ28" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ28" t="inlineStr">
+      <c r="BR28" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR28" t="inlineStr">
+      <c r="BS28" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS28" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT28" t="inlineStr">
+      <c r="BT28" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU28" t="inlineStr">
         <is>
           <t>alcohol/1-s2.0-S2589537025000811-main (1).pdf</t>
         </is>
@@ -8351,62 +8491,67 @@
       </c>
       <c r="BG29" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH29" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH29" t="inlineStr">
+      <c r="BI29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI29" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ29" t="n">
         <v>0</v>
       </c>
       <c r="BK29" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL29" t="n">
         <v>40</v>
       </c>
-      <c r="BL29" t="inlineStr">
+      <c r="BM29" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM29" t="inlineStr">
+      <c r="BN29" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN29" t="inlineStr">
+      <c r="BO29" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO29" t="inlineStr">
+      <c r="BP29" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP29" t="inlineStr">
+      <c r="BQ29" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ29" t="inlineStr">
+      <c r="BR29" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR29" t="inlineStr">
+      <c r="BS29" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS29" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT29" t="inlineStr">
+      <c r="BT29" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU29" t="inlineStr">
         <is>
           <t>alcohol/115d425e-5129-48c5-8c21-e1af10229ed5 (1).pdf</t>
         </is>
@@ -8617,62 +8762,67 @@
       </c>
       <c r="BG30" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH30" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH30" t="inlineStr">
+      <c r="BI30" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI30" t="n">
+      <c r="BJ30" t="n">
         <v>2</v>
       </c>
-      <c r="BJ30" t="n">
-        <v>1</v>
-      </c>
       <c r="BK30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL30" t="n">
         <v>4</v>
       </c>
-      <c r="BL30" t="inlineStr">
+      <c r="BM30" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM30" t="inlineStr">
+      <c r="BN30" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN30" t="inlineStr">
+      <c r="BO30" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO30" t="inlineStr">
+      <c r="BP30" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP30" t="inlineStr">
+      <c r="BQ30" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ30" t="inlineStr">
+      <c r="BR30" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR30" t="inlineStr">
+      <c r="BS30" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS30" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT30" t="inlineStr">
+      <c r="BT30" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU30" t="inlineStr">
         <is>
           <t>alcohol/bcr-2019-230109 (1).pdf</t>
         </is>
@@ -8881,64 +9031,69 @@
       </c>
       <c r="BG31" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH31" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH31" t="inlineStr">
+      <c r="BI31" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI31" t="n">
+      <c r="BJ31" t="n">
         <v>3</v>
       </c>
-      <c r="BJ31" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK31" t="n">
+      <c r="BK31" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL31" t="n">
         <v>14</v>
       </c>
-      <c r="BL31" t="inlineStr">
+      <c r="BM31" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM31" t="inlineStr">
+      <c r="BN31" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN31" t="inlineStr">
+      <c r="BO31" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO31" t="inlineStr">
+      <c r="BP31" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP31" t="inlineStr">
+      <c r="BQ31" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ31" t="inlineStr">
+      <c r="BR31" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR31" t="inlineStr">
+      <c r="BS31" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS31" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT31" t="inlineStr">
+      <c r="BT31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU31" t="inlineStr">
         <is>
           <t>alcohol/BIMA_Paper_for_Pure (1).pdf</t>
         </is>
@@ -9157,68 +9312,73 @@
       </c>
       <c r="BG32" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BH32" t="inlineStr">
+        <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BH32" t="inlineStr">
+      <c r="BI32" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BI32" t="inlineStr">
+      <c r="BJ32" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BJ32" t="inlineStr">
+      <c r="BK32" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BK32" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BL32" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM32" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM32" t="inlineStr">
+      <c r="BN32" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BN32" t="inlineStr">
+      <c r="BO32" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO32" t="inlineStr">
+      <c r="BP32" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP32" t="inlineStr">
+      <c r="BQ32" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ32" t="inlineStr">
+      <c r="BR32" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR32" t="inlineStr">
+      <c r="BS32" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS32" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT32" t="inlineStr">
+      <c r="BT32" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU32" t="inlineStr">
         <is>
           <t>alcohol/Smart, R. G., &amp; Storm, T. (1964). The efficacy of LSD in the treatment of alcoholism.pdf</t>
         </is>
@@ -9439,62 +9599,67 @@
       </c>
       <c r="BG33" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH33" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH33" t="inlineStr">
+      <c r="BI33" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI33" t="n">
-        <v>1</v>
-      </c>
       <c r="BJ33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK33" t="n">
         <v>2</v>
       </c>
-      <c r="BK33" t="n">
+      <c r="BL33" t="n">
         <v>30</v>
       </c>
-      <c r="BL33" t="inlineStr">
+      <c r="BM33" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM33" t="inlineStr">
+      <c r="BN33" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN33" t="inlineStr">
+      <c r="BO33" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO33" t="inlineStr">
+      <c r="BP33" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP33" t="inlineStr">
+      <c r="BQ33" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ33" t="inlineStr">
+      <c r="BR33" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR33" t="inlineStr">
+      <c r="BS33" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS33" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT33" t="inlineStr">
+      <c r="BT33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU33" t="inlineStr">
         <is>
           <t>alcohol/1966_smart_4543_1 (1).pdf</t>
         </is>
@@ -9705,64 +9870,69 @@
       </c>
       <c r="BG34" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH34" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH34" t="inlineStr">
+      <c r="BI34" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI34" t="n">
+      <c r="BJ34" t="n">
         <v>5</v>
       </c>
-      <c r="BJ34" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK34" t="n">
+      <c r="BK34" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL34" t="n">
         <v>24</v>
       </c>
-      <c r="BL34" t="inlineStr">
+      <c r="BM34" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM34" t="inlineStr">
+      <c r="BN34" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN34" t="inlineStr">
+      <c r="BO34" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO34" t="inlineStr">
+      <c r="BP34" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP34" t="inlineStr">
+      <c r="BQ34" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ34" t="inlineStr">
+      <c r="BR34" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR34" t="inlineStr">
+      <c r="BS34" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS34" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT34" t="inlineStr">
+      <c r="BT34" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU34" t="inlineStr">
         <is>
           <t>alcohol/Smith, C. M. (1958). A new adjunct to the treatment of alcoholism The hallucinogenic drugs.pdf</t>
         </is>
@@ -9973,64 +10143,69 @@
       </c>
       <c r="BG35" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH35" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH35" t="inlineStr">
+      <c r="BI35" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI35" t="n">
+      <c r="BJ35" t="n">
         <v>43</v>
       </c>
-      <c r="BJ35" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK35" t="n">
+      <c r="BK35" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL35" t="n">
         <v>13</v>
       </c>
-      <c r="BL35" t="inlineStr">
+      <c r="BM35" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM35" t="inlineStr">
+      <c r="BN35" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN35" t="inlineStr">
+      <c r="BO35" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO35" t="inlineStr">
+      <c r="BP35" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP35" t="inlineStr">
+      <c r="BQ35" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ35" t="inlineStr">
+      <c r="BR35" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR35" t="inlineStr">
+      <c r="BS35" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS35" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT35" t="inlineStr">
+      <c r="BT35" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU35" t="inlineStr">
         <is>
           <t>alcohol/s13722-022-00345-y (1).pdf</t>
         </is>
@@ -10241,24 +10416,24 @@
       </c>
       <c r="BG36" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH36" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH36" t="inlineStr">
+      <c r="BI36" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI36" t="inlineStr">
+      <c r="BJ36" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ36" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BK36" t="inlineStr">
         <is>
           <t>.</t>
@@ -10266,43 +10441,48 @@
       </c>
       <c r="BL36" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM36" t="inlineStr">
+        <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM36" t="inlineStr">
+      <c r="BN36" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN36" t="inlineStr">
+      <c r="BO36" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO36" t="inlineStr">
+      <c r="BP36" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP36" t="inlineStr">
+      <c r="BQ36" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ36" t="inlineStr">
+      <c r="BR36" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR36" t="inlineStr">
+      <c r="BS36" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS36" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT36" t="inlineStr">
+      <c r="BT36" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU36" t="inlineStr">
         <is>
           <t>alcohol/agaf031 (1).pdf</t>
         </is>
@@ -10515,66 +10695,71 @@
       </c>
       <c r="BG37" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH37" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH37" t="inlineStr">
+      <c r="BI37" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI37" t="n">
+      <c r="BJ37" t="n">
         <v>3</v>
       </c>
-      <c r="BJ37" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BK37" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL37" t="inlineStr">
+        <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BL37" t="inlineStr">
+      <c r="BM37" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM37" t="inlineStr">
+      <c r="BN37" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN37" t="inlineStr">
+      <c r="BO37" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO37" t="inlineStr">
+      <c r="BP37" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP37" t="inlineStr">
+      <c r="BQ37" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ37" t="inlineStr">
+      <c r="BR37" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR37" t="inlineStr">
+      <c r="BS37" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS37" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT37" t="inlineStr">
+      <c r="BT37" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU37" t="inlineStr">
         <is>
           <t>alcohol/qjsa.1970.31.932.pdf</t>
         </is>
@@ -10791,64 +10976,69 @@
       </c>
       <c r="BG38" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BH38" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH38" t="inlineStr">
+      <c r="BI38" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI38" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ38" t="n">
         <v>0</v>
       </c>
-      <c r="BK38" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
+      <c r="BK38" t="n">
+        <v>0</v>
       </c>
       <c r="BL38" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BM38" t="inlineStr">
+        <is>
           <t>NA</t>
         </is>
       </c>
-      <c r="BM38" t="inlineStr">
+      <c r="BN38" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN38" t="inlineStr">
+      <c r="BO38" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO38" t="inlineStr">
+      <c r="BP38" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP38" t="inlineStr">
+      <c r="BQ38" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ38" t="inlineStr">
+      <c r="BR38" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR38" t="inlineStr">
+      <c r="BS38" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS38" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT38" t="inlineStr">
+      <c r="BT38" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU38" t="inlineStr">
         <is>
           <t>alcohol/s12888-024-05502-y (1).pdf</t>
         </is>
@@ -11057,62 +11247,67 @@
       </c>
       <c r="BG39" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH39" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH39" t="inlineStr">
+      <c r="BI39" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI39" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ39" t="n">
         <v>0</v>
       </c>
       <c r="BK39" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL39" t="n">
         <v>5</v>
       </c>
-      <c r="BL39" t="inlineStr">
+      <c r="BM39" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM39" t="inlineStr">
+      <c r="BN39" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN39" t="inlineStr">
+      <c r="BO39" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO39" t="inlineStr">
+      <c r="BP39" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP39" t="inlineStr">
+      <c r="BQ39" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ39" t="inlineStr">
+      <c r="BR39" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR39" t="inlineStr">
+      <c r="BS39" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS39" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT39" t="inlineStr">
+      <c r="BT39" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU39" t="inlineStr">
         <is>
           <t>alcohol/jamapsychiatry.2018.3990.pdf</t>
         </is>
@@ -11329,62 +11524,67 @@
       </c>
       <c r="BG40" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH40" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH40" t="inlineStr">
+      <c r="BI40" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="BI40" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ40" t="n">
         <v>0</v>
       </c>
       <c r="BK40" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL40" t="n">
         <v>27</v>
       </c>
-      <c r="BL40" t="inlineStr">
+      <c r="BM40" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM40" t="inlineStr">
+      <c r="BN40" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="BN40" t="inlineStr">
+      <c r="BO40" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO40" t="inlineStr">
+      <c r="BP40" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP40" t="inlineStr">
+      <c r="BQ40" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ40" t="inlineStr">
+      <c r="BR40" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR40" t="inlineStr">
+      <c r="BS40" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS40" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT40" t="inlineStr">
+      <c r="BT40" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU40" t="inlineStr">
         <is>
           <t>opioids/j.1749-6632.2000.tb05213.x.pdf</t>
         </is>
@@ -11597,62 +11797,67 @@
       </c>
       <c r="BG41" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH41" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH41" t="inlineStr">
+      <c r="BI41" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI41" t="n">
+      <c r="BJ41" t="n">
         <v>4</v>
       </c>
-      <c r="BJ41" t="n">
+      <c r="BK41" t="n">
         <v>5</v>
       </c>
-      <c r="BK41" t="n">
+      <c r="BL41" t="n">
         <v>45</v>
       </c>
-      <c r="BL41" t="inlineStr">
+      <c r="BM41" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM41" t="inlineStr">
+      <c r="BN41" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN41" t="inlineStr">
+      <c r="BO41" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO41" t="inlineStr">
+      <c r="BP41" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP41" t="inlineStr">
+      <c r="BQ41" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ41" t="inlineStr">
+      <c r="BR41" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR41" t="inlineStr">
+      <c r="BS41" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS41" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT41" t="inlineStr">
+      <c r="BT41" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU41" t="inlineStr">
         <is>
           <t>opioids/Jovaisa et al.pdf</t>
         </is>
@@ -11865,62 +12070,67 @@
       </c>
       <c r="BG42" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH42" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH42" t="inlineStr">
+      <c r="BI42" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI42" t="n">
-        <v>1</v>
-      </c>
       <c r="BJ42" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="BK42" t="n">
         <v>70</v>
       </c>
-      <c r="BL42" t="inlineStr">
+      <c r="BL42" t="n">
+        <v>70</v>
+      </c>
+      <c r="BM42" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM42" t="inlineStr">
+      <c r="BN42" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN42" t="inlineStr">
+      <c r="BO42" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO42" t="inlineStr">
+      <c r="BP42" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP42" t="inlineStr">
+      <c r="BQ42" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ42" t="inlineStr">
+      <c r="BR42" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR42" t="inlineStr">
+      <c r="BS42" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS42" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT42" t="inlineStr">
+      <c r="BT42" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU42" t="inlineStr">
         <is>
           <t>opioids/PIIS0740547202002751.pdf</t>
         </is>
@@ -12131,62 +12341,67 @@
       </c>
       <c r="BG43" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH43" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH43" t="inlineStr">
+      <c r="BI43" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI43" t="n">
-        <v>1</v>
-      </c>
       <c r="BJ43" t="n">
-        <v>59</v>
+        <v>1</v>
       </c>
       <c r="BK43" t="n">
         <v>59</v>
       </c>
-      <c r="BL43" t="inlineStr">
+      <c r="BL43" t="n">
+        <v>59</v>
+      </c>
+      <c r="BM43" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM43" t="inlineStr">
+      <c r="BN43" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN43" t="inlineStr">
+      <c r="BO43" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO43" t="inlineStr">
+      <c r="BP43" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP43" t="inlineStr">
+      <c r="BQ43" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ43" t="inlineStr">
+      <c r="BR43" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR43" t="inlineStr">
+      <c r="BS43" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS43" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT43" t="inlineStr">
+      <c r="BT43" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU43" t="inlineStr">
         <is>
           <t>opioids/02791072.2007.10399860.pdf</t>
         </is>
@@ -12395,64 +12610,69 @@
       </c>
       <c r="BG44" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH44" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH44" t="inlineStr">
+      <c r="BI44" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI44" t="inlineStr">
+      <c r="BJ44" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ44" t="n">
+      <c r="BK44" t="n">
         <v>22</v>
       </c>
-      <c r="BK44" t="n">
+      <c r="BL44" t="n">
         <v>27</v>
       </c>
-      <c r="BL44" t="inlineStr">
+      <c r="BM44" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM44" t="inlineStr">
+      <c r="BN44" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN44" t="inlineStr">
+      <c r="BO44" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO44" t="inlineStr">
+      <c r="BP44" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP44" t="inlineStr">
+      <c r="BQ44" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ44" t="inlineStr">
+      <c r="BR44" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR44" t="inlineStr">
+      <c r="BS44" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS44" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT44" t="inlineStr">
+      <c r="BT44" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU44" t="inlineStr">
         <is>
           <t>opioids/Ascending_single_dose_double_blind_place.pdf</t>
         </is>
@@ -12648,79 +12868,84 @@
       </c>
       <c r="BD45" t="inlineStr">
         <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="BE45" t="inlineStr">
+        <is>
+          <t>out_of_scope_substance</t>
+        </is>
+      </c>
+      <c r="BF45" t="inlineStr">
+        <is>
+          <t>Randomized double-blind trial reporting substance-use outcomes (criteria a and b met), but all 20 patients were enrolled for DSM-IV cocaine dependence and every outcome (Minnesota Cocaine Craving Scale, cocaine-positive urine screens) concerns cocaine use. No tobacco, alcohol, or opioid endpoint is reported. Fails criterion (c): out of the review scope.</t>
+        </is>
+      </c>
+      <c r="BG45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH45" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BE45" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="BF45" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
-      <c r="BG45" t="inlineStr">
+      <c r="BI45" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH45" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="BI45" t="n">
-        <v>1</v>
-      </c>
-      <c r="BJ45" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK45" t="n">
+      <c r="BJ45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK45" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL45" t="n">
         <v>10</v>
       </c>
-      <c r="BL45" t="inlineStr">
+      <c r="BM45" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM45" t="inlineStr">
+      <c r="BN45" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN45" t="inlineStr">
+      <c r="BO45" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO45" t="inlineStr">
+      <c r="BP45" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP45" t="inlineStr">
+      <c r="BQ45" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ45" t="inlineStr">
+      <c r="BR45" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR45" t="inlineStr">
+      <c r="BS45" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS45" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT45" t="inlineStr">
+      <c r="BT45" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU45" t="inlineStr">
         <is>
           <t>opioids/Ibogaine_Effect_on_Cocaine_Craving_and_U.pdf</t>
         </is>
@@ -12931,66 +13156,71 @@
       </c>
       <c r="BG46" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH46" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH46" t="inlineStr">
+      <c r="BI46" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI46" t="n">
+      <c r="BJ46" t="n">
         <v>3</v>
       </c>
-      <c r="BJ46" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
       <c r="BK46" t="inlineStr">
         <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL46" t="inlineStr">
+        <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BL46" t="inlineStr">
+      <c r="BM46" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM46" t="inlineStr">
+      <c r="BN46" t="inlineStr">
         <is>
           <t>Severe</t>
         </is>
       </c>
-      <c r="BN46" t="inlineStr">
+      <c r="BO46" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO46" t="inlineStr">
+      <c r="BP46" t="inlineStr">
         <is>
           <t>text</t>
         </is>
       </c>
-      <c r="BP46" t="inlineStr">
+      <c r="BQ46" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ46" t="inlineStr">
+      <c r="BR46" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR46" t="inlineStr">
+      <c r="BS46" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS46" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT46" t="inlineStr">
+      <c r="BT46" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU46" t="inlineStr">
         <is>
           <t>opioids/archpsyc.1973.01750360040005.pdf</t>
         </is>
@@ -13203,62 +13433,67 @@
       </c>
       <c r="BG47" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH47" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH47" t="inlineStr">
+      <c r="BI47" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI47" t="n">
-        <v>1</v>
-      </c>
       <c r="BJ47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK47" t="n">
         <v>6</v>
       </c>
-      <c r="BK47" t="n">
+      <c r="BL47" t="n">
         <v>15</v>
       </c>
-      <c r="BL47" t="inlineStr">
+      <c r="BM47" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM47" t="inlineStr">
+      <c r="BN47" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN47" t="inlineStr">
+      <c r="BO47" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO47" t="inlineStr">
+      <c r="BP47" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP47" t="inlineStr">
+      <c r="BQ47" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ47" t="inlineStr">
+      <c r="BR47" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR47" t="inlineStr">
+      <c r="BS47" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS47" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT47" t="inlineStr">
+      <c r="BT47" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU47" t="inlineStr">
         <is>
           <t>smoking/nihms-648744.pdf</t>
         </is>
@@ -13469,64 +13704,69 @@
       </c>
       <c r="BG48" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH48" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH48" t="inlineStr">
+      <c r="BI48" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI48" t="n">
+      <c r="BJ48" t="n">
         <v>3</v>
       </c>
-      <c r="BJ48" t="inlineStr">
-        <is>
-          <t>.</t>
-        </is>
-      </c>
-      <c r="BK48" t="n">
+      <c r="BK48" t="inlineStr">
+        <is>
+          <t>.</t>
+        </is>
+      </c>
+      <c r="BL48" t="n">
         <v>15</v>
       </c>
-      <c r="BL48" t="inlineStr">
+      <c r="BM48" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM48" t="inlineStr">
+      <c r="BN48" t="inlineStr">
         <is>
           <t>Mild</t>
         </is>
       </c>
-      <c r="BN48" t="inlineStr">
+      <c r="BO48" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO48" t="inlineStr">
+      <c r="BP48" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP48" t="inlineStr">
+      <c r="BQ48" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ48" t="inlineStr">
+      <c r="BR48" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR48" t="inlineStr">
+      <c r="BS48" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS48" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT48" t="inlineStr">
+      <c r="BT48" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU48" t="inlineStr">
         <is>
           <t>smoking/nihms648730.pdf</t>
         </is>
@@ -13739,62 +13979,67 @@
       </c>
       <c r="BG49" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH49" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH49" t="inlineStr">
+      <c r="BI49" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI49" t="n">
-        <v>1</v>
-      </c>
       <c r="BJ49" t="n">
         <v>1</v>
       </c>
       <c r="BK49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BL49" t="n">
         <v>15</v>
       </c>
-      <c r="BL49" t="inlineStr">
+      <c r="BM49" t="inlineStr">
         <is>
           <t>psychedelic_arm</t>
         </is>
       </c>
-      <c r="BM49" t="inlineStr">
+      <c r="BN49" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN49" t="inlineStr">
+      <c r="BO49" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO49" t="inlineStr">
+      <c r="BP49" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP49" t="inlineStr">
+      <c r="BQ49" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ49" t="inlineStr">
+      <c r="BR49" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR49" t="inlineStr">
+      <c r="BS49" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS49" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT49" t="inlineStr">
+      <c r="BT49" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU49" t="inlineStr">
         <is>
           <t>smoking/johnson2016.pdf</t>
         </is>
@@ -14005,64 +14250,69 @@
       </c>
       <c r="BG50" t="inlineStr">
         <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="BH50" t="inlineStr">
+        <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BH50" t="inlineStr">
+      <c r="BI50" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="BI50" t="inlineStr">
+      <c r="BJ50" t="inlineStr">
         <is>
           <t>Not numbered</t>
         </is>
       </c>
-      <c r="BJ50" t="n">
+      <c r="BK50" t="n">
         <v>70</v>
       </c>
-      <c r="BK50" t="n">
+      <c r="BL50" t="n">
         <v>82</v>
       </c>
-      <c r="BL50" t="inlineStr">
+      <c r="BM50" t="inlineStr">
         <is>
           <t>pooled</t>
         </is>
       </c>
-      <c r="BM50" t="inlineStr">
+      <c r="BN50" t="inlineStr">
         <is>
           <t>Moderate</t>
         </is>
       </c>
-      <c r="BN50" t="inlineStr">
+      <c r="BO50" t="inlineStr">
         <is>
           <t>born-digital</t>
         </is>
       </c>
-      <c r="BO50" t="inlineStr">
+      <c r="BP50" t="inlineStr">
         <is>
           <t>markdown</t>
         </is>
       </c>
-      <c r="BP50" t="inlineStr">
+      <c r="BQ50" t="inlineStr">
         <is>
           <t>claude-sonnet-5</t>
         </is>
       </c>
-      <c r="BQ50" t="inlineStr">
+      <c r="BR50" t="inlineStr">
         <is>
           <t>v1.2</t>
         </is>
       </c>
-      <c r="BR50" t="inlineStr">
+      <c r="BS50" t="inlineStr">
         <is>
           <t>v1</t>
         </is>
       </c>
-      <c r="BS50" t="n">
-        <v>1</v>
-      </c>
-      <c r="BT50" t="inlineStr">
+      <c r="BT50" t="n">
+        <v>1</v>
+      </c>
+      <c r="BU50" t="inlineStr">
         <is>
           <t>smoking/johnson_2026_oi_260062_1772564464.70221 (1).pdf</t>
         </is>

</xml_diff>